<commit_message>
fullgame/FG-M1: FG1-SIG-05 核心固件迁移与 AI 边界
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/fg/#FirmwareKind-固件种类.xlsx
+++ b/Configs/GameConfig/Datas/fg/#FirmwareKind-固件种类.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,7 +569,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>regular</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>regular</t>
+          <t>core</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -621,6 +621,90 @@
       </c>
       <c r="E9" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>fw_capacitor</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>firmware.fw_capacitor.name</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>fw_swarm</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>firmware.fw_swarm.name</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>fw_amplify</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>firmware.fw_amplify.name</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fw_execute</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>firmware.fw_execute.name</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>